<commit_message>
slicing & fetching "data user: nakes", update import kader
</commit_message>
<xml_diff>
--- a/public/template_data_kader.xlsx
+++ b/public/template_data_kader.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\lapor-mas-mantri\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A140AF-63DC-4413-9F91-6E0DEBADA945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC28D06-F2DC-470B-9F1B-FDE6D9B564BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1980" yWindow="3110" windowWidth="17220" windowHeight="8170" xr2:uid="{AD5913CA-9426-40E6-A57B-02F1265C700D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AD5913CA-9426-40E6-A57B-02F1265C700D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,27 +36,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
-    <t>nama</t>
-  </si>
-  <si>
-    <t>username</t>
-  </si>
-  <si>
-    <t>nama_kelurahan</t>
-  </si>
-  <si>
-    <t>nama_posyandu</t>
-  </si>
-  <si>
-    <t>no_telepon</t>
-  </si>
-  <si>
-    <t>jenis_kelamin</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
     <t>Siti Aminah</t>
   </si>
   <si>
@@ -82,6 +61,27 @@
   </si>
   <si>
     <t>kader_ana</t>
+  </si>
+  <si>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Nama Kelurahan</t>
+  </si>
+  <si>
+    <t>Nama Posyandu</t>
+  </si>
+  <si>
+    <t>No Telepon</t>
+  </si>
+  <si>
+    <t>Jenis Kelamin</t>
   </si>
 </sst>
 </file>
@@ -456,71 +456,71 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>123456</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F2">
         <v>8123456789</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>123456</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F3">
         <v>8123456789</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change to fetchwithauth (dashboard, kelola user, data wilayah)
</commit_message>
<xml_diff>
--- a/public/template_data_kader.xlsx
+++ b/public/template_data_kader.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\lapor-mas-mantri\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC28D06-F2DC-470B-9F1B-FDE6D9B564BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B715825-3F12-49CD-AD65-0AB774326724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AD5913CA-9426-40E6-A57B-02F1265C700D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Siti Aminah</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Jenis Kelamin</t>
+  </si>
+  <si>
+    <t>08123456789</t>
   </si>
 </sst>
 </file>
@@ -125,9 +128,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,7 +457,7 @@
     <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -493,10 +500,10 @@
       <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="F2">
-        <v>8123456789</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
@@ -516,10 +523,10 @@
       <c r="E3" t="s">
         <v>4</v>
       </c>
-      <c r="F3">
-        <v>8123456789</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>